<commit_message>
Fix FAISS index: embed full 100K pool with all-MiniLM-L6-v2, exact flat search retrieval, improve title gating and active signals
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -441,1800 +441,1800 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8092</v>
+        <v>0.8347</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Demonstrated 5.9 YOE in engineering as Senior AI Engineer at Apple. Shipped: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Lists skills: FAISS, PINECONE. Experience with A/B TEST, system evaluation.</t>
+          <t>6y Senior Machine Learning Engineer at Genpact AI. Key achievement: Led the migration from keyword-based to embedding-based search across a 30M+ candidate corpus over 8 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0070202</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6862</v>
+        <v>0.7803</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.1 years experience as Machine Learning Engineer at BYJU'S. Shipped key systems: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Lists skills: QDRANT. Experience with A/B TEST evaluation.</t>
+          <t>16y Senior Applied Scientist at Meta. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0092255</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6365</v>
+        <v>0.7739</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.2 years experience as ML Engineer at InMobi. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: WEAVIATE, OPENSEARCH. Experience with evaluation.</t>
+          <t>7y Lead AI Engineer at Razorpay. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0010603</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6015</v>
+        <v>0.7695</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Proven track record with 5.3 YOE as ML Engineer at BYJU'S. Key work: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: PGVECTOR, OPENSEARCH.</t>
+          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0019288</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.601</v>
+        <v>0.7582</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Proven track record with 5.7 YOE as AI Research Engineer at Paytm. Key work: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. Lists skills: FAISS, PGVECTOR.</t>
+          <t>7y Senior Machine Learning Engineer at Zomato. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0001819</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5943000000000001</v>
+        <v>0.7396</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Proven track record with 4.4 YOE as ML Engineer at Genpact AI. Key work: Built models in Prophet, LightGBM, and (for one project) a small LSTM — the LightGBM model ended up shipping. Lists skills: WEAVIATE, PGVECTOR.</t>
+          <t>8y Search Engineer at Sarvam AI. Key achievement: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0042100</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.578</v>
+        <v>0.7333</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Proven track record with 7.3 YOE as Machine Learning Engineer at Freshworks. Key work: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Lists skills: PINECONE, ELASTICSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>6y Senior AI Engineer at Apple. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0083637</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.575</v>
+        <v>0.7332</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Demonstrated 3.4 YOE in engineering as ML Engineer at Unacademy. Shipped: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard.</t>
+          <t>5y AI Engineer at Mad Street Den. Key achievement: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0099751</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5711000000000001</v>
+        <v>0.7284</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Proven track record with 5.5 YOE as Junior ML Engineer at Observe.AI. Key work: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: WEAVIATE.</t>
+          <t>7y AI Engineer at Google. Key achievement: Developed a semantic search feature for an internal knowledge base of ~500K documents. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0043829</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.5685</v>
+        <v>0.7272999999999999</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Observe.AI with 4.8 YOE. Handled systems involving Machine Learning, Qdrant, Go. Lists skills: QDRANT.</t>
+          <t>8y Senior AI Engineer at Netflix. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0074648</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5651</v>
+        <v>0.7222</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4.1 years experience as AI Research Engineer at Flipkart. Shipped key systems: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: QDRANT, PINECONE. Experience with evaluation.</t>
+          <t>Applied ML Engineer at Sarvam AI (6.6 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0070485</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5603</v>
+        <v>0.7219</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Demonstrated 6.4 YOE in engineering as Search Engineer at Saarthi.ai. Shipped: Developed a semantic search feature for an internal knowledge base of ~500K documents. Shipped systems using FAISS, ELASTICSEARCH. Experience with evaluation.</t>
+          <t>AI Engineer at Flipkart (16.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0061696</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.5602</v>
+        <v>0.711</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Background as Senior Software Engineer (ML) at Glance with 3.5 YOE, with expertise in Speech Recognition, Microservices, pgvector. Lists skills: PINECONE, WEAVIATE.</t>
+          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0040117</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5601</v>
+        <v>0.705</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Proven track record with 6.5 YOE as Recommendation Systems Engineer at PhonePe. Key work: Built a content recommendation system serving 10M+ users that combined collaborative filtering with content-based ranking. Shipped systems using PINECONE. Experience with A/B TEST, system evaluation.</t>
+          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5564</v>
+        <v>0.6995</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.7 years experience as AI Research Engineer at Haptik. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: MILVUS, QDRANT.</t>
+          <t>Senior Machine Learning Engineer at Flipkart (8.1 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0049540</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.555</v>
+        <v>0.6911</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Proven track record with 6.8 YOE as ML Engineer at Saarthi.ai. Key work: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: PGVECTOR. Experience with evaluation.</t>
+          <t>Search Engineer at CRED (5.1 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0073556</t>
+          <t>CAND_0040887</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.5457</v>
+        <v>0.6873</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Nykaa with 4.4 YOE. Handled systems involving Image Classification, LlamaIndex, Forecasting. Lists skills: QDRANT.</t>
+          <t>Machine Learning Engineer at Netflix (4.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0097896</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5423</v>
+        <v>0.6833</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Demonstrated 4.8 YOE in engineering as AI Research Engineer at upGrad. Shipped: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: MILVUS, QDRANT. Experience with evaluation.</t>
+          <t>Senior AI Engineer at Meta (7.9 YOE). Notable: Built systems that understand what users are looking for and connect them to the most relevant matches across a large dataset. JD alignment: embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0043958</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.5377999999999999</v>
+        <v>0.6667</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6.7 years experience as AI Research Engineer at Dream11. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: FAISS. Experience with evaluation.</t>
+          <t>AI Engineer at CRED (16.9 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0067609</t>
+          <t>CAND_0053591</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5364</v>
+        <v>0.6661</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Proven track record with 4.5 YOE as Junior ML Engineer at Wysa. Key work: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: QDRANT. Experience with evaluation.</t>
+          <t>AI Engineer at Ola (5.3 YOE). Notable: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0039838</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.5341</v>
+        <v>0.6636</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Proven track record with 4.9 YOE as Recommendation Systems Engineer at Amazon. Key work: Built and operated production ML pipelines using MLflow for experiment tracking, Kubeflow for orchestration, and our internal feature store. Shipped systems using FAISS. Experience with A/B TEST, system evaluation.</t>
+          <t>Senior Applied Scientist at Sarvam AI (5.3 YOE). Notable: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0064130</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.5312</v>
+        <v>0.6601</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>6.7 years experience as AI Research Engineer at Unacademy. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production.</t>
+          <t>AI Engineer at Rephrase.ai (6.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0037117</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5289</v>
+        <v>0.6506999999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Proven track record with 4.6 YOE as Computer Vision Engineer at Mad Street Den. Key work: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard.</t>
+          <t>AI Engineer at PolicyBazaar (7.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0021491</t>
+          <t>CAND_0058575</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.5212</v>
+        <v>0.6124000000000001</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6.1 years experience as AI Research Engineer at Wysa. Shipped key systems: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. Lists skills: ELASTICSEARCH.</t>
+          <t>AI Engineer at Krutrim (5.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0052712</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.5143</v>
+        <v>0.6119</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.1 years experience as AI Research Engineer at Verloop.io. Shipped key systems: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard.</t>
+          <t>Machine Learning Engineer at BYJU'S (4.5 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0060340</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.494</v>
+        <v>0.6115</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Proven track record with 6.1 YOE as Computer Vision Engineer at Wysa. Key work: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: PGVECTOR.</t>
+          <t>Applied ML Engineer at CRED (5.1 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0073418</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.4916</v>
+        <v>0.6095</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer at Niramai with 3.0 YOE. Handled systems involving Machine Learning, Weights &amp; Biases, Diffusion Models. Lists skills: OPENSEARCH.</t>
+          <t>Search Engineer at Verloop.io (4.2 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0065450</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.4735</v>
+        <v>0.6085</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.0 years experience as ML Engineer at Tech Mahindra. Shipped key systems: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: PINECONE. Experience with evaluation.</t>
+          <t>Lead AI Engineer at Sarvam AI (6.4 YOE). Notable: Owned the search and discovery experience end-to-end at a consumer product, from how content is represented internally through to how the most rele... JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0008049</t>
+          <t>CAND_0043381</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4704</v>
+        <v>0.6001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Demonstrated 6.3 YOE in engineering as ML Engineer at Niramai. Shipped: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Experience with evaluation.</t>
+          <t>AI Research Engineer at PharmEasy (3.6 YOE). Notable: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0037290</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.4701</v>
+        <v>0.5959</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Worked as Computer Vision Engineer at InMobi (3.2 YOE) focusing on systems for TensorFlow, Object Detection, OpenCV.</t>
+          <t>Senior AI Engineer at Adobe (5.9 YOE). Notable: Led the engineering team building infrastructure to surface relevant content to users at scale. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0088335</t>
+          <t>CAND_0018888</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.4549</v>
+        <v>0.5949</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Demonstrated 6.4 YOE in engineering as AI Research Engineer at Tech Mahindra. Shipped: Built models in Prophet, LightGBM, and (for one project) a small LSTM — the LightGBM model ended up shipping. Lists skills: WEAVIATE. Experience with evaluation.</t>
+          <t>AI Research Engineer at Razorpay, 6.5 years. Skills: pgvector, GANs, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0094916</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.453</v>
+        <v>0.5889</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3.7 years experience as Junior ML Engineer at Tech Mahindra. Shipped key systems: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: PGVECTOR. Experience with evaluation.</t>
+          <t>Search Engineer at Haptik, 5.2 years. Skills: Computer Vision, Semantic Search, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0067091</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.449</v>
+        <v>0.5863</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4.8 years experience as Senior Software Engineer (ML) at Saarthi.ai. Shipped key systems: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: FAISS, PINECONE. Experience with evaluation.</t>
+          <t>AI Engineer at PharmEasy, 5.9 years. Skills: Python, Elasticsearch, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0091229</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.4461</v>
+        <v>0.5857</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>7.0 years experience as Senior Software Engineer (ML) at Niramai. Shipped key systems: Built models in Prophet, LightGBM, and (for one project) a small LSTM — the LightGBM model ended up shipping. Lists skills: FAISS, QDRANT.</t>
+          <t>AI Engineer at Mad Street Den, 6.3 years. Skills: Embeddings, TensorFlow, PyTorch. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0085557</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.4368</v>
+        <v>0.5856</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Demonstrated 3.1 YOE in engineering as Data Scientist at Rephrase.ai. Shipped: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: WEAVIATE, PGVECTOR.</t>
+          <t>Search Engineer at Google, 7.2 years. Skills: LoRA, PyTorch, QLoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0069643</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.4345</v>
+        <v>0.5745</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Proven track record with 7.1 YOE as Senior Software Engineer at Vedantu. Key work: Built the company's first proper data warehouse (migrating from a tangled set of Postgres replicas to a clean Snowflake setup with dbt), the... Lists skills: MILVUS.</t>
+          <t>Search Engineer at Haptik, 7.6 years. Skills: Hugging Face Transformers, Image Classification, Forecasting. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0069953</t>
+          <t>CAND_0084819</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.4208</v>
+        <v>0.5651</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5.4 years experience as Computer Vision Engineer at Wipro. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: OPENSEARCH, ELASTICSEARCH.</t>
+          <t>Search Engineer at Dream11, 4.5 years. Skills: LoRA, Semantic Search, BM25. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0002637</t>
+          <t>CAND_0004402</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.4061</v>
+        <v>0.5604</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Demonstrated 4.4 YOE in engineering as Senior Software Engineer at PhonePe. Shipped: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Yellow.ai, 6.0 years. Skills: PEFT, BentoML, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Delhi, Delhi, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0077798</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.4051</v>
+        <v>0.5547</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8.0 years experience as Software Engineer at Meesho. Shipped key systems: Built our experimentation framework that supports the product team's A/B tests. Lists skills: WEAVIATE. Experience with A/B TEST evaluation.</t>
+          <t>Senior Data Scientist at Sarvam AI, 7.4 years. Skills: Information Retrieval, QLoRA, RAG. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0060715</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.3991</v>
+        <v>0.548</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Proven track record with 3.3 YOE as ML Engineer at Genpact AI. Key work: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: FAISS.</t>
+          <t>Lead AI Engineer at Meta, 8.6 years. Skills: scikit-learn, NLP, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0030207</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.3766</v>
+        <v>0.5451</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Demonstrated 4.0 YOE in engineering as Data Scientist at PhonePe. Shipped: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: PGVECTOR, ELASTICSEARCH.</t>
+          <t>Senior Data Scientist at Niramai, 5.2 years. Skills: OpenSearch, Semantic Search, LlamaIndex. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0071977</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.3712</v>
+        <v>0.5445</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Proven track record with 3.6 YOE as Senior Data Engineer at PharmEasy. Key work: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards. Lists skills: PINECONE.</t>
+          <t>Search Engineer at CRED, 7.8 years. Skills: Weaviate, Python, scikit-learn. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0023307</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.3674</v>
+        <v>0.5419</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Demonstrated 5.2 YOE in engineering as Senior Software Engineer at Cognizant. Shipped: Built and maintained data pipelines on Apache Airflow processing ~500GB of daily transactional data across 12 source systems. Experience with A/B TEST evaluation.</t>
+          <t>Machine Learning Engineer at Genpact AI, 7.2 years. Skills: BM25, Data Science, LoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0049116</t>
+          <t>CAND_0076831</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.3628</v>
+        <v>0.5401</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Demonstrated 7.7 YOE in engineering as Senior Data Engineer at Freshworks. Shipped: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>Search Engineer at Krutrim, 4.0 years. Skills: Milvus, BM25, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0031366</t>
+          <t>CAND_0022023</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.3477</v>
+        <v>0.5373</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Proven track record with 3.3 YOE as Data Engineer at Swiggy. Key work: Built our experimentation framework that supports the product team's A/B tests. Lists skills: MILVUS, PGVECTOR. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Saarthi.ai, 4.6 years. Skills: Machine Learning, Time Series, Diffusion Models. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Pune, Maharashtra, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0039386</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.3454</v>
+        <v>0.5372</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.4 years experience as Senior Data Engineer at CRED. Shipped key systems: Built our experimentation framework that supports the product team's A/B tests. Lists skills: FAISS, PGVECTOR. Experience with A/B TEST evaluation.</t>
+          <t>Senior NLP Engineer at Mad Street Den, 8.0 years. Skills: Milvus, LlamaIndex, TensorFlow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Vizag, Andhra Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0015306</t>
+          <t>CAND_0020708</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.3444</v>
+        <v>0.5325</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Demonstrated 4.3 YOE in engineering as Senior Data Engineer at Unacademy. Shipped: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: ELASTICSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>Search Engineer at PolicyBazaar, 4.2 years. Skills: scikit-learn, LLMs, TensorFlow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Indore, Madhya Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0076225</t>
+          <t>CAND_0001610</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.3422</v>
+        <v>0.5315</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Proven track record with 3.8 YOE as Software Engineer at Paytm. Key work: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: PINECONE. Experience with A/B TEST evaluation.</t>
+          <t>Machine Learning Engineer at Dream11, 3.0 years. Skills: scikit-learn, Speech Recognition, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0054453</t>
+          <t>CAND_0092278</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.3415</v>
+        <v>0.5308</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Demonstrated 7.8 YOE in engineering as Senior Data Engineer at Wipro. Shipped: Built and maintained data pipelines on Apache Airflow processing ~500GB of daily transactional data across 12 source systems. Lists skills: WEAVIATE.</t>
+          <t>Senior NLP Engineer at Microsoft, 6.8 years. Skills: TensorFlow, QLoRA, Time Series. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0051507</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.3398</v>
+        <v>0.529</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Demonstrated 4.6 YOE in engineering as Senior Software Engineer at BYJU'S. Shipped: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards. Lists skills: QDRANT, OPENSEARCH.</t>
+          <t>AI Engineer at Mad Street Den, 6.4 years. Skills: TensorFlow, Recommendation Systems, FAISS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0039824</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.3355</v>
+        <v>0.5262</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>3.2 years experience as Senior Software Engineer at InMobi. Shipped key systems: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>NLP Engineer at Krutrim, 5.2 years. Skills: Python, RAG, Time Series. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Chennai, Tamil Nadu, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0084090</t>
+          <t>CAND_0035879</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.3317</v>
+        <v>0.5155</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Demonstrated 3.9 YOE in engineering as Junior ML Engineer at Ola. Shipped: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: QDRANT, PGVECTOR. Experience with evaluation.</t>
+          <t>AI Research Engineer at Krutrim, 4.5 years. Skills: Speech Recognition, Diffusion Models, Python. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0039587</t>
+          <t>CAND_0041611</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.3299</v>
+        <v>0.5068</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>6.2 years experience as Data Engineer at HCL. Shipped key systems: Built our experimentation framework that supports the product team's A/B tests. Lists skills: WEAVIATE. Experience with A/B TEST evaluation.</t>
+          <t>Staff Machine Learning Engineer at Locobuzz, 6.4 years. Skills: LangChain, OpenSearch, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0098815</t>
+          <t>CAND_0079830</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.328</v>
+        <v>0.4987</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Proven track record with 6.4 YOE as Senior Data Engineer at PharmEasy. Key work: Built our experimentation framework that supports the product team's A/B tests. Lists skills: QDRANT. Experience with A/B TEST evaluation.</t>
+          <t>Junior ML Engineer at BYJU'S, 3.6 years. Skills: Computer Vision, MLOps, Data Science. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0042761</t>
+          <t>CAND_0076995</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.3214</v>
+        <v>0.4911</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>5.2 years experience as Senior Software Engineer at Mphasis. Shipped key systems: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers. Lists skills: FAISS, MILVUS.</t>
+          <t>AI Research Engineer at Haptik, 4.4 years. Skills: Reinforcement Learning, Prompt Engineering, scikit-learn. Partial JD fit on search/ranking/retrieval systems, production ML system deployment.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0079900</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.3208</v>
+        <v>0.4903</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Proven track record with 7.2 YOE as Senior Data Engineer at PolicyBazaar. Key work: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers.</t>
+          <t>Senior Data Scientist at Rephrase.ai, 5.7 years. Skills: Recommendation Systems, Forecasting, Haystack. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0006437</t>
+          <t>CAND_0063585</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.3207</v>
+        <v>0.49</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>6.2 years experience as Senior Software Engineer (ML) at Razorpay. Shipped key systems: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. Lists skills: OPENSEARCH.</t>
+          <t>AI Research Engineer at Observe.AI, 3.1 years. Skills: Learning to Rank, MLflow, Reinforcement Learning. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0050539</t>
+          <t>CAND_0070485</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.3182</v>
+        <v>0.4893</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Proven track record with 5.1 YOE as Software Engineer at Accenture. Key work: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: FAISS.</t>
+          <t>Search Engineer at Saarthi.ai, 6.4 years. Skills: QLoRA, Deep Learning, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0025738</t>
+          <t>CAND_0034169</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.3171</v>
+        <v>0.4785</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Proven track record with 5.4 YOE as Senior Software Engineer at Razorpay. Key work: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers. Lists skills: OPENSEARCH.</t>
+          <t>AI Research Engineer at Krutrim, 3.4 years. Skills: Hugging Face Transformers, Diffusion Models, Fine-tuning LLMs. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0080187</t>
+          <t>CAND_0080315</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.3163</v>
+        <v>0.4768</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Demonstrated 6.2 YOE in engineering as Senior Data Engineer at Swiggy. Shipped: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers.</t>
+          <t>AI Research Engineer at Sarvam AI, 4.1 years. Skills: Diffusion Models, LangChain, Image Classification. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Ahmedabad, Gujarat, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0029614</t>
+          <t>CAND_0022852</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.3161</v>
+        <v>0.4755</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Proven track record with 5.3 YOE as Backend Engineer at Dream11. Key work: Built the company's first proper data warehouse (migrating from a tangled set of Postgres replicas to a clean Snowflake setup with dbt), the... Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Zomato (5.4 YOE). Skills: Weights &amp; Biases, OpenCV, Python.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0044046</t>
+          <t>CAND_0021827</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.3143</v>
+        <v>0.467</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Demonstrated 5.9 YOE in engineering as Senior Software Engineer at upGrad. Shipped: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform.</t>
+          <t>AI Research Engineer at Unacademy (4.4 YOE). Skills: Weights &amp; Biases, Object Detection, Diffusion Models.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0008589</t>
+          <t>CAND_0016170</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.3133</v>
+        <v>0.465</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Demonstrated 6.8 YOE in engineering as Software Engineer at Flipkart. Shipped: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: WEAVIATE.</t>
+          <t>AI Research Engineer at Dream11 (6.8 YOE). Skills: Time Series, Reinforcement Learning, Hugging Face Transformers. Logistics friction: 90-day notice (standard); work mode: flexible.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0012459</t>
+          <t>CAND_0097472</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.3131</v>
+        <v>0.4556</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Demonstrated 6.6 YOE in engineering as Senior Software Engineer at Meesho. Shipped: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards.</t>
+          <t>Junior ML Engineer at Flipkart (5.8 YOE). Skills: CNN, Information Retrieval, YOLO.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0034914</t>
+          <t>CAND_0087316</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.3113</v>
+        <v>0.4548</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Demonstrated 3.5 YOE in engineering as Senior Software Engineer at Paytm. Shipped: Built and maintained data pipelines on Apache Airflow processing ~500GB of daily transactional data across 12 source systems.</t>
+          <t>AI Research Engineer at Razorpay (4.1 YOE). Skills: Speech Recognition, NLP, CNN.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0043119</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.3096</v>
+        <v>0.4501</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Demonstrated 3.6 YOE in engineering as Software Engineer at Meesho. Shipped: Built our experimentation framework that supports the product team's A/B tests. Lists skills: OPENSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Haptik (6.7 YOE). Skills: Qdrant, Recommendation Systems, Python.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0063138</t>
+          <t>CAND_0064331</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.3086</v>
+        <v>0.4467</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Demonstrated 7.2 YOE in engineering as Analytics Engineer at Zoho. Shipped: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers. Lists skills: PGVECTOR, OPENSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>Senior Software Engineer (ML) at Swiggy (4.2 YOE). Skills: Forecasting, Data Science, YOLO.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0073669</t>
+          <t>CAND_0049771</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.3072</v>
+        <v>0.4389</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Proven track record with 4.3 YOE as Senior Software Engineer at Ola. Key work: Built the company's first proper data warehouse (migrating from a tangled set of Postgres replicas to a clean Snowflake setup with dbt), the... Lists skills: PGVECTOR.</t>
+          <t>AI Research Engineer at Wysa (5.0 YOE). Skills: Python, ASR, OpenCV.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0034876</t>
+          <t>CAND_0046526</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.3067</v>
+        <v>0.431</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Proven track record with 3.5 YOE as Computer Vision Engineer at InMobi. Key work: Built models in Prophet, LightGBM, and (for one project) a small LSTM — the LightGBM model ended up shipping. Lists skills: PGVECTOR, OPENSEARCH.</t>
+          <t>ML Engineer at Ola (5.5 YOE). Skills: FAISS, Time Series, Weights &amp; Biases.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0051165</t>
+          <t>CAND_0039308</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.3061</v>
+        <v>0.4298</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Demonstrated 6.2 YOE in engineering as Analytics Engineer at Zomato. Shipped: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: PGVECTOR, OPENSEARCH.</t>
+          <t>AI Research Engineer at BYJU'S (5.6 YOE). Skills: Time Series, OpenSearch, Haystack. Logistics friction: long 120-day notice period; work mode: hybrid.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0082447</t>
+          <t>CAND_0008517</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.3052</v>
+        <v>0.4275</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Proven track record with 5.4 YOE as Analytics Engineer at Freshworks. Key work: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Locobuzz (5.6 YOE). Skills: Feature Engineering, PyTorch, Weights &amp; Biases.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0069059</t>
+          <t>CAND_0065139</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.3037</v>
+        <v>0.4258</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>6.4 years experience as Senior Software Engineer at BYJU'S. Shipped key systems: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers. Lists skills: MILVUS.</t>
+          <t>AI Research Engineer at Niramai (5.2 YOE). Skills: LangChain, MLOps, Speech Recognition.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0000131</t>
+          <t>CAND_0022415</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.303</v>
+        <v>0.4225</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>4.8 years experience as Data Analyst at upGrad. Shipped key systems: Built the company's first proper data warehouse (migrating from a tangled set of Postgres replicas to a clean Snowflake setup with dbt), the... Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Observe.AI (3.2 YOE). Skills: OpenCV, Prompt Engineering, Image Classification.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0000010</t>
+          <t>CAND_0014858</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.301</v>
+        <v>0.4057</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Proven track record with 4.6 YOE as Data Engineer at Ola. Key work: Built our experimentation framework that supports the product team's A/B tests. Lists skills: ELASTICSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Aganitha (4.9 YOE). Skills: Time Series, Diffusion Models, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0000158</t>
+          <t>CAND_0093185</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.299</v>
+        <v>0.4003</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>4.4 years experience as Frontend Engineer at Stark Industries. Shipped key systems: Built the company's design system from scratch and led the migration from a legacy AngularJS app. Lists skills: ELASTICSEARCH.</t>
+          <t>AI Research Engineer at Dream11 (4.1 YOE). Skills: Forecasting, LoRA, YOLO. Logistics friction: long 120-day notice period; work mode: flexible.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0073224</t>
+          <t>CAND_0018925</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.2986</v>
+        <v>0.3972</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Demonstrated 4.4 YOE in engineering as Data Engineer at Paytm. Shipped: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Rephrase.ai (5.8 YOE). Skills: Haystack, Speech Recognition, Deep Learning. Logistics friction: 90-day notice (standard); work mode: remote.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0089195</t>
+          <t>CAND_0069248</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.2962</v>
+        <v>0.3969</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4.2 years experience as Senior Data Engineer at BYJU'S. Shipped key systems: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards.</t>
+          <t>AI Research Engineer at Unacademy (5.4 YOE). Skills: OpenCV, QLoRA, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0022943</t>
+          <t>CAND_0000422</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.2941</v>
+        <v>0.3912</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>6.0 years experience as Senior Data Engineer at Freshworks. Shipped key systems: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers.</t>
+          <t>AI Research Engineer at Haptik (6.3 YOE). Skills: Python, OpenCV, Reinforcement Learning.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0000014</t>
+          <t>CAND_0051219</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.294</v>
+        <v>0.385</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>8.4 years experience as Frontend Engineer at Zomato. Shipped key systems: Built the company's design system from scratch and led the migration from a legacy AngularJS app. Lists skills: FAISS, OPENSEARCH.</t>
+          <t>AI Research Engineer at Observe.AI (3.8 YOE). Skills: Reinforcement Learning, YOLO, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0002403</t>
+          <t>CAND_0085557</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.2938</v>
+        <v>0.3719</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Demonstrated 4.4 YOE in engineering as Senior Data Engineer at Zomato. Shipped: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform.</t>
+          <t>Data Scientist at Rephrase.ai (3.1 YOE). Skills: Feature Engineering, Machine Learning, RAG.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0000043</t>
+          <t>CAND_0073007</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.293</v>
+        <v>0.3677</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Proven track record with 8.3 YOE as Cloud Engineer at Swiggy. Key work: Built and maintained the end-to-end test suite using Selenium and pytest, plus the load-testing setup using Locust. Lists skills: OPENSEARCH, ELASTICSEARCH.</t>
+          <t>AI Specialist at Aganitha, 5.8 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: MLflow, Speech Recognition, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0021800</t>
+          <t>CAND_0041625</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.2894</v>
+        <v>0.3435</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>6.0 years experience as Software Engineer at PharmEasy. Shipped key systems: Built our experimentation framework that supports the product team's A/B tests. Experience with A/B TEST evaluation.</t>
+          <t>AI Research Engineer at Infosys, 4.7 years. Ranked lower due to: not actively job-seeking. Has: Object Detection, FAISS, Statistical Modeling.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0009232</t>
+          <t>CAND_0025046</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2884</v>
+        <v>0.3038</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Proven track record with 4.0 YOE as Senior Software Engineer at Tech Mahindra. Key work: Owned the analytics-and-reporting service which serves dashboards to ~3K paying customers. Lists skills: WEAVIATE.</t>
+          <t>AI Specialist at Genpact AI, 6.7 years. Ranked lower due to: not actively job-seeking. Has: TTS, Object Detection, Embeddings.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0000155</t>
+          <t>CAND_0016267</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.287</v>
+        <v>0.2869</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>3.2 years experience as Software Engineer at Unacademy. Shipped key systems: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards. Lists skills: MILVUS.</t>
+          <t>AI Specialist at Freshworks, 3.6 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: YOLO, PyTorch, Information Retrieval.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0091367</t>
+          <t>CAND_0075922</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.2853</v>
+        <v>0.282</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>4.5 years experience as Senior Software Engineer at Swiggy. Shipped key systems: Built and maintained data pipelines on Apache Airflow processing ~500GB of daily transactional data across 12 source systems. Lists skills: QDRANT, ELASTICSEARCH.</t>
+          <t>Customer Support at Wipro, 12.8 years. Ranked lower due to: not actively job-seeking. Has: Airflow, Sales, FastAPI.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0072362</t>
+          <t>CAND_0070653</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.2789</v>
+        <v>0.2815</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>5.7 years experience as Analytics Engineer at Unacademy. Shipped key systems: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards. Lists skills: MILVUS. Experience with A/B TEST evaluation.</t>
+          <t>AI Specialist at Dream11, 5.0 years. Ranked lower due to: not actively job-seeking. Has: PyTorch, Sentence Transformers, Kubeflow.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0096314</t>
+          <t>CAND_0062264</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2784</v>
+        <v>0.2751</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>7.9 years experience as Software Engineer at HCL. Shipped key systems: Designed and maintained the analytical data warehouse on Snowflake supporting the BI team's ~50 dashboards. Experience with A/B TEST evaluation.</t>
+          <t>Customer Support at Acme Corp, 11.5 years. Ranked lower due to: low recruiter engagement; not actively job-seeking. Has: Next.js, gRPC, Sales.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0095457</t>
+          <t>CAND_0009236</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.278</v>
+        <v>0.2737</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Demonstrated 4.1 YOE in engineering as Data Scientist at Locobuzz. Shipped: Built computer vision models for our product's image moderation feature using PyTorch — fine-tuned ResNet variants on a labeled dataset of ~200K... Lists skills: MILVUS, WEAVIATE. Experience with evaluation.</t>
+          <t>AI Specialist at Vedantu, 6.3 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: LangChain, Speech Recognition, Learning to Rank.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0000031</t>
+          <t>CAND_0062784</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.275</v>
+        <v>0.2689</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Proven track record with 6.0 YOE as Recommendation Systems Engineer at Swiggy. Key work: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Lists skills: FAISS, PINECONE. Experience with A/B TEST, system evaluation.</t>
+          <t>Customer Support at Dunder Mifflin, 8.0 years. Ranked lower due to: weak production ML systems evidence; not actively job-seeking. Has: Salesforce CRM, Next.js, Tailwind.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0000160</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.275</v>
+        <v>0.2665</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Proven track record with 7.0 YOE as Software Engineer at Zomato. Key work: Built and maintained the end-to-end test suite using Selenium and pytest, plus the load-testing setup using Locust. Lists skills: ELASTICSEARCH.</t>
+          <t>AI Specialist at Aganitha, 5.9 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: LLMs, Fine-tuning LLMs, Forecasting.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0000001</t>
+          <t>CAND_0096612</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.274</v>
+        <v>0.2657</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Proven track record with 6.9 YOE as Backend Engineer at Mindtree. Key work: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform. Lists skills: MILVUS.</t>
+          <t>Customer Support at Initech, 9.1 years. Ranked lower due to: long notice (120d). Has: TTS, dbt, Redux.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0000097</t>
+          <t>CAND_0096103</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.273</v>
+        <v>0.2619</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Proven track record with 5.8 YOE as Mechanical Engineer at TCS. Key work: Owned the demand-generation function — content marketing, paid acquisition, SEO, email nurture. Lists skills: FAISS, PINECONE.</t>
+          <t>Customer Support at TCS, 7.6 years. Ranked lower due to: low recruiter engagement. Has: Java, Six Sigma, Flask.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0093958</t>
+          <t>CAND_0075469</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2713</v>
+        <v>0.2616</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Proven track record with 5.9 YOE as Junior ML Engineer at Meesho. Key work: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. Lists skills: FAISS.</t>
+          <t>Customer Support at Pied Piper, 5.4 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Tally, TypeScript, Excel.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0000187</t>
+          <t>CAND_0025354</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.271</v>
+        <v>0.2608</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Proven track record with 6.6 YOE as DevOps Engineer at Mphasis. Key work: Built React-based admin interfaces and the Node.</t>
+          <t>Customer Support at Hooli, 4.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Microservices, Scrum, gRPC.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0009101</t>
+          <t>CAND_0003840</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.269</v>
+        <v>0.2569</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>5.9 years experience as Analytics Engineer at Cognizant. Shipped key systems: Implemented streaming data pipelines on Kafka and Spark Streaming for a real-time user-activity processing platform.</t>
+          <t>Customer Support at Wipro, 10.6 years. Ranked lower due to: not actively job-seeking. Has: Object Detection, Spring Boot, gRPC.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0043089</t>
+          <t>CAND_0046955</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2656</v>
+        <v>0.255</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Demonstrated 4.7 YOE in engineering as Data Engineer at Paytm. Shipped: Built our experimentation framework that supports the product team's A/B tests. Lists skills: PINECONE. Experience with A/B TEST evaluation.</t>
+          <t>Customer Support at Dunder Mifflin, 14.3 years. Ranked lower due to: long notice (120d); logistics mismatch; not actively job-seeking. Has: Azure, MongoDB, Angular.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0068256</t>
+          <t>CAND_0016663</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2655</v>
+        <v>0.2515</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Demonstrated 4.5 YOE in engineering as Cloud Engineer at Swiggy. Shipped: Built React-based admin interfaces and the Node. Lists skills: PINECONE.</t>
+          <t>Customer Support at Dunder Mifflin, 4.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Accounting, gRPC, Vue.js.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0094564</t>
+          <t>CAND_0017831</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2652</v>
+        <v>0.2514</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Proven track record with 5.1 YOE as Analytics Engineer at Nykaa. Key work: Built the company's first proper data warehouse (migrating from a tangled set of Postgres replicas to a clean Snowflake setup with dbt), the... Lists skills: OPENSEARCH. Experience with A/B TEST evaluation.</t>
+          <t>Customer Support at Initech, 3.5 years. Ranked lower due to: not actively job-seeking. Has: Time Series, Snowflake, gRPC.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0093682</t>
+          <t>CAND_0046766</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2646</v>
+        <v>0.2496</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Proven track record with 4.1 YOE as Data Engineer at Razorpay. Key work: Built our experimentation framework that supports the product team's A/B tests. Lists skills: PINECONE, WEAVIATE. Experience with A/B TEST evaluation.</t>
+          <t>Customer Support at TCS, 10.8 years. Ranked lower due to: not actively job-seeking. Has: Docker, Webpack, Go.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0000015</t>
+          <t>CAND_0088602</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.259</v>
+        <v>0.2482</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Demonstrated 5.4 YOE in engineering as Software Engineer at Razorpay. Shipped: Owned the AWS account architecture (VPC, IAM, networking), the Terraform modules for our service deployments, and the Kubernetes cluster operations. Lists skills: QDRANT.</t>
+          <t>AI Specialist at Niramai, 4.8 years. Ranked lower due to: logistics mismatch. Has: TensorFlow, Feature Engineering, Semantic Search.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Increase REDUCED_POOL_SIZE to 12000, tighten MISMATCH_TITLES, and rebuild the exact nearest-neighbor search to produce a clean Top-100 list with zero customer support/accounting profiles
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -466,7 +466,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7803</v>
+        <v>0.7701</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -477,36 +477,36 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7739</v>
+        <v>0.7694</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7y Lead AI Engineer at Razorpay. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7695</v>
+        <v>0.768</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Lead AI Engineer at Razorpay. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7582</v>
+        <v>0.7578</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -531,18 +531,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7396</v>
+        <v>0.749</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8y Search Engineer at Sarvam AI. Key achievement: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Staff Machine Learning Engineer at Paytm. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7333</v>
+        <v>0.7276</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -567,1674 +567,1674 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7332</v>
+        <v>0.7164</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5y AI Engineer at Mad Street Den. Key achievement: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>8y Senior AI Engineer at Netflix. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7284</v>
+        <v>0.7122000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7y AI Engineer at Google. Key achievement: Developed a semantic search feature for an internal knowledge base of ~500K documents. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Applied ML Engineer at Sarvam AI. Key achievement: Developed a semantic search feature for an internal knowledge base of ~500K documents. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7272999999999999</v>
+        <v>0.7116</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8y Senior AI Engineer at Netflix. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>5y AI Engineer at Mad Street Den. Key achievement: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.7222</v>
+        <v>0.7084</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Sarvam AI (6.6 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Flipkart (16.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.7219</v>
+        <v>0.707</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AI Engineer at Flipkart (16.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Google (7.3 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0005260</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.711</v>
+        <v>0.7046</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.705</v>
+        <v>0.7030999999999999</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0064326</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.6995</v>
+        <v>0.7012</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer at Flipkart (8.1 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Sarvam AI (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6911</v>
+        <v>0.6956</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Search Engineer at CRED (5.1 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior Machine Learning Engineer at Flipkart (8.1 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0040887</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.6873</v>
+        <v>0.6862</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Netflix (4.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Niramai (7.8 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0006567</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6833</v>
+        <v>0.6764</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Meta (7.9 YOE). Notable: Built systems that understand what users are looking for and connect them to the most relevant matches across a large dataset. JD alignment: embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>Search Engineer at CRED (5.1 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0040887</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.6667</v>
+        <v>0.6709000000000001</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI Engineer at CRED (16.9 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Machine Learning Engineer at Netflix (4.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0053591</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.6661</v>
+        <v>0.6606</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AI Engineer at Ola (5.3 YOE). Notable: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior Applied Scientist at Sarvam AI (5.3 YOE). Notable: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.6636</v>
+        <v>0.6583</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist at Sarvam AI (5.3 YOE). Notable: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at CRED (16.9 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0098846</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.6601</v>
+        <v>0.6554</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Engineer at Rephrase.ai (6.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at upGrad (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.6506999999999999</v>
+        <v>0.6475</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Engineer at PolicyBazaar (7.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Ola (7.8 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0058575</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.6124000000000001</v>
+        <v>0.6348</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AI Engineer at Krutrim (5.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Junior ML Engineer at Aganitha (6.1 YOE). Notable: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0030348</t>
+          <t>CAND_0053591</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6119</v>
+        <v>0.6338</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at BYJU'S (4.5 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Ola (5.3 YOE). Notable: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0020877</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.6115</v>
+        <v>0.6335</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at CRED (5.1 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Rephrase.ai (6.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.6095</v>
+        <v>0.6316000000000001</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Search Engineer at Verloop.io (4.2 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at PolicyBazaar (7.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0068351</t>
+          <t>CAND_0006567</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.6085</v>
+        <v>0.631</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Lead AI Engineer at Sarvam AI (6.4 YOE). Notable: Owned the search and discovery experience end-to-end at a consumer product, from how content is represented internally through to how the most rele... JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Senior AI Engineer at Meta (7.9 YOE). Notable: Built systems that understand what users are looking for and connect them to the most relevant matches across a large dataset. JD alignment: embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0043381</t>
+          <t>CAND_0043637</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6001</v>
+        <v>0.6099</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AI Research Engineer at PharmEasy (3.6 YOE). Notable: Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at FAANG, but production. JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Junior ML Engineer at Rephrase.ai (5.5 YOE). Notable: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0005538</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.5959</v>
+        <v>0.6051</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Adobe (5.9 YOE). Notable: Led the engineering team building infrastructure to surface relevant content to users at scale. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Rephrase.ai (4.2 YOE). Notable: Built a content recommendation system serving 10M+ users that combined collaborative filtering with content-based ranking. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0018888</t>
+          <t>CAND_0030348</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.5949</v>
+        <v>0.5994</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Razorpay, 6.5 years. Skills: pgvector, GANs, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Machine Learning Engineer at BYJU'S, 4.5 years. Skills: pgvector, GANs, Vector Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Noida, Uttar Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0041568</t>
+          <t>CAND_0020877</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5889</v>
+        <v>0.5921</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Search Engineer at Haptik, 5.2 years. Skills: Computer Vision, Semantic Search, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Applied ML Engineer at CRED, 5.1 years. Skills: PyTorch, YOLO, Qdrant. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0081686</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.5863</v>
+        <v>0.5895</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>AI Engineer at PharmEasy, 5.9 years. Skills: Python, Elasticsearch, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Netflix, 6.0 years. Skills: Python, Milvus, Kubeflow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Austin, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0044883</t>
+          <t>CAND_0042506</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.5857</v>
+        <v>0.5865</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AI Engineer at Mad Street Den, 6.3 years. Skills: Embeddings, TensorFlow, PyTorch. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>Search Engineer at Verloop.io, 4.2 years. Skills: NLP, Forecasting, FAISS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Mumbai, Maharashtra, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0028793</t>
+          <t>CAND_0058575</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.5856</v>
+        <v>0.586</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Search Engineer at Google, 7.2 years. Skills: LoRA, PyTorch, QLoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
+          <t>AI Engineer at Krutrim, 5.8 years. Skills: Hugging Face Transformers, Sentence Transformers, Reinforcement Learning. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0076251</t>
+          <t>CAND_0030468</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.5745</v>
+        <v>0.5854</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Search Engineer at Haptik, 7.6 years. Skills: Hugging Face Transformers, Image Classification, Forecasting. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior Applied Scientist at Swiggy, 5.4 years. Skills: Search &amp; Discovery, Text Encoders, Content Matching. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0084819</t>
+          <t>CAND_0054318</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.5651</v>
+        <v>0.57</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Search Engineer at Dream11, 4.5 years. Skills: LoRA, Semantic Search, BM25. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Research Engineer at BYJU'S, 3.5 years. Skills: GANs, Diffusion Models, LoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Chandigarh, Chandigarh, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0004402</t>
+          <t>CAND_0045250</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.5604</v>
+        <v>0.5675</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Yellow.ai, 6.0 years. Skills: PEFT, BentoML, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Delhi, Delhi, not open to relocation.</t>
+          <t>Applied ML Engineer at Rephrase.ai, 6.6 years. Skills: Sentence Transformers, NLP, PEFT. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Delhi, Delhi, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0005649</t>
+          <t>CAND_0005538</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5547</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Sarvam AI, 7.4 years. Skills: Information Retrieval, QLoRA, RAG. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>Senior AI Engineer at Adobe, 5.9 years. Skills: Information Retrieval Systems, TTS, pgvector. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0018888</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.548</v>
+        <v>0.5654</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Lead AI Engineer at Meta, 8.6 years. Skills: scikit-learn, NLP, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Research Engineer at Razorpay, 6.5 years. Skills: pgvector, GANs, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0079064</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.5451</v>
+        <v>0.5646</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Niramai, 5.2 years. Skills: OpenSearch, Semantic Search, LlamaIndex. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at PharmEasy, 5.9 years. Skills: Python, Elasticsearch, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0083307</t>
+          <t>CAND_0041568</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5445</v>
+        <v>0.5643</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Search Engineer at CRED, 7.8 years. Skills: Weaviate, Python, scikit-learn. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Haptik, 5.2 years. Skills: Computer Vision, Semantic Search, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0070398</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5419</v>
+        <v>0.5636</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Genpact AI, 7.2 years. Skills: BM25, Data Science, LoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
+          <t>AI Engineer at Mad Street Den, 6.3 years. Skills: Embeddings, TensorFlow, PyTorch. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0076831</t>
+          <t>CAND_0094056</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.5401</v>
+        <v>0.5585</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Search Engineer at Krutrim, 4.0 years. Skills: Milvus, BM25, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>NLP Engineer at Rephrase.ai, 5.9 years. Skills: Sentence Transformers, Embeddings, LlamaIndex. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0022023</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.5373</v>
+        <v>0.5563</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Saarthi.ai, 4.6 years. Skills: Machine Learning, Time Series, Diffusion Models. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Pune, Maharashtra, not open to relocation.</t>
+          <t>Search Engineer at Haptik, 7.6 years. Skills: Hugging Face Transformers, Image Classification, Forecasting. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5372</v>
+        <v>0.5534</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Mad Street Den, 8.0 years. Skills: Milvus, LlamaIndex, TensorFlow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Vizag, Andhra Pradesh, not open to relocation.</t>
+          <t>Machine Learning Engineer at BYJU'S, 5.1 years. Skills: BM25, RAG, Weights &amp; Biases. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0020708</t>
+          <t>CAND_0028793</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5325</v>
+        <v>0.5516</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Search Engineer at PolicyBazaar, 4.2 years. Skills: scikit-learn, LLMs, TensorFlow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Indore, Madhya Pradesh, not open to relocation.</t>
+          <t>Search Engineer at Google, 7.2 years. Skills: LoRA, PyTorch, QLoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0001610</t>
+          <t>CAND_0080766</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.5315</v>
+        <v>0.5502</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Dream11, 3.0 years. Skills: scikit-learn, Speech Recognition, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>Staff Machine Learning Engineer at Salesforce, 8.8 years. Skills: OpenSearch, Deep Learning, Search Infrastructure. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0068351</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5308</v>
+        <v>0.5473</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Microsoft, 6.8 years. Skills: TensorFlow, QLoRA, Time Series. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Lead AI Engineer at Sarvam AI, 6.4 years. Skills: PEFT, Deep Learning, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Delhi, Delhi, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.529</v>
+        <v>0.5461</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>AI Engineer at Mad Street Den, 6.4 years. Skills: TensorFlow, Recommendation Systems, FAISS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior Data Scientist at Sarvam AI, 7.4 years. Skills: Information Retrieval, QLoRA, RAG. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0096172</t>
+          <t>CAND_0036437</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.5262</v>
+        <v>0.5436</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>NLP Engineer at Krutrim, 5.2 years. Skills: Python, RAG, Time Series. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Chennai, Tamil Nadu, not open to relocation.</t>
+          <t>Search Engineer at Rephrase.ai, 4.8 years. Skills: FAISS, Milvus, Vector Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0035879</t>
+          <t>CAND_0052335</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.5155</v>
+        <v>0.5423</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Krutrim, 4.5 years. Skills: Speech Recognition, Diffusion Models, Python. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Applied ML Engineer at Aganitha, 6.4 years. Skills: Learning to Rank, GANs, Sentence Transformers. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.5068</v>
+        <v>0.5423</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Locobuzz, 6.4 years. Skills: LangChain, OpenSearch, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Lead AI Engineer at Meta, 8.6 years. Skills: scikit-learn, NLP, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0079830</t>
+          <t>CAND_0051004</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.4987</v>
+        <v>0.5417999999999999</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Junior ML Engineer at BYJU'S, 3.6 years. Skills: Computer Vision, MLOps, Data Science. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Logistics concern: long 120-day notice period.</t>
+          <t>Senior Data Scientist at CRED, 4.7 years. Skills: Prompt Engineering, LlamaIndex, Semantic Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0076995</t>
+          <t>CAND_0025640</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.4911</v>
+        <v>0.5403</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Haptik, 4.4 years. Skills: Reinforcement Learning, Prompt Engineering, scikit-learn. Partial JD fit on search/ranking/retrieval systems, production ML system deployment.</t>
+          <t>AI Research Engineer at HCL, 5.6 years. Skills: Elasticsearch, CNN, Semantic Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Jaipur, Rajasthan, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0029367</t>
+          <t>CAND_0046132</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.4903</v>
+        <v>0.5387</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Rephrase.ai, 5.7 years. Skills: Recommendation Systems, Forecasting, Haystack. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Research Engineer at Verloop.io, 4.3 years. Skills: Time Series, MLflow, MLOps. Partial JD fit on search/ranking/retrieval systems, production ML system deployment. Based in Noida, Uttar Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0063585</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.49</v>
+        <v>0.5356</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Observe.AI, 3.1 years. Skills: Learning to Rank, MLflow, Reinforcement Learning. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
+          <t>Applied ML Engineer at Saarthi.ai, 5.8 years. Skills: Elasticsearch, Milvus, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Jaipur, Rajasthan, not open to relocation.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0070485</t>
+          <t>CAND_0084819</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.4893</v>
+        <v>0.5328000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Search Engineer at Saarthi.ai, 6.4 years. Skills: QLoRA, Deep Learning, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Dream11, 4.5 years. Skills: LoRA, Semantic Search, BM25. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0034169</t>
+          <t>CAND_0015065</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.4785</v>
+        <v>0.5325</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Krutrim, 3.4 years. Skills: Hugging Face Transformers, Diffusion Models, Fine-tuning LLMs. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>AI Research Engineer at Flipkart, 3.9 years. Skills: Learning to Rank, LlamaIndex, Information Retrieval. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0080315</t>
+          <t>CAND_0018722</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.4768</v>
+        <v>0.5306999999999999</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Sarvam AI, 4.1 years. Skills: Diffusion Models, LangChain, Image Classification. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Ahmedabad, Gujarat, not open to relocation.</t>
+          <t>Recommendation Systems Engineer at Saarthi.ai, 6.6 years. Skills: TensorFlow, GANs, Hugging Face Transformers. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0022852</t>
+          <t>CAND_0033861</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.4755</v>
+        <v>0.53</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Zomato (5.4 YOE). Skills: Weights &amp; Biases, OpenCV, Python.</t>
+          <t>Senior NLP Engineer at Mad Street Den (8.0 YOE). Skills: Milvus, LlamaIndex, TensorFlow.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0021827</t>
+          <t>CAND_0015578</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.467</v>
+        <v>0.5292</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Unacademy (4.4 YOE). Skills: Weights &amp; Biases, Object Detection, Diffusion Models.</t>
+          <t>AI Engineer at Zoho (5.4 YOE). Skills: Machine Learning, Speech Recognition, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0016170</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.465</v>
+        <v>0.5283</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Dream11 (6.8 YOE). Skills: Time Series, Reinforcement Learning, Hugging Face Transformers. Logistics friction: 90-day notice (standard); work mode: flexible.</t>
+          <t>Search Engineer at PharmEasy (5.2 YOE). Skills: Sentence Transformers, NLP, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0097472</t>
+          <t>CAND_0008295</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.4556</v>
+        <v>0.5236</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Junior ML Engineer at Flipkart (5.8 YOE). Skills: CNN, Information Retrieval, YOLO.</t>
+          <t>AI Research Engineer at Razorpay (6.5 YOE). Skills: QLoRA, Python, BentoML.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0087316</t>
+          <t>CAND_0092278</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.4548</v>
+        <v>0.5225</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Razorpay (4.1 YOE). Skills: Speech Recognition, NLP, CNN.</t>
+          <t>Senior NLP Engineer at Microsoft (6.8 YOE). Skills: TensorFlow, QLoRA, Time Series.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.4501</v>
+        <v>0.5207000000000001</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Haptik (6.7 YOE). Skills: Qdrant, Recommendation Systems, Python.</t>
+          <t>Senior Software Engineer (ML) at Mad Street Den (5.4 YOE). Skills: Statistical Modeling, Python, LLMs.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0064331</t>
+          <t>CAND_0043381</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.4467</v>
+        <v>0.5177</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) at Swiggy (4.2 YOE). Skills: Forecasting, Data Science, YOLO.</t>
+          <t>AI Research Engineer at PharmEasy (3.6 YOE). Skills: Forecasting, scikit-learn, OpenSearch.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0079064</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.4389</v>
+        <v>0.5155</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Wysa (5.0 YOE). Skills: Python, ASR, OpenCV.</t>
+          <t>Senior Data Scientist at Niramai (5.2 YOE). Skills: OpenSearch, Semantic Search, LlamaIndex.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0046526</t>
+          <t>CAND_0083879</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.431</v>
+        <v>0.5103</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ML Engineer at Ola (5.5 YOE). Skills: FAISS, Time Series, Weights &amp; Biases.</t>
+          <t>Machine Learning Engineer at Ola (7.1 YOE). Skills: Hugging Face Transformers, Prompt Engineering, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0039308</t>
+          <t>CAND_0083307</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.4298</v>
+        <v>0.5099</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>AI Research Engineer at BYJU'S (5.6 YOE). Skills: Time Series, OpenSearch, Haystack. Logistics friction: long 120-day notice period; work mode: hybrid.</t>
+          <t>Search Engineer at CRED (7.8 YOE). Skills: Weaviate, Python, scikit-learn. Logistics friction: long 120-day notice period; work mode: flexible.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0008517</t>
+          <t>CAND_0072232</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.4275</v>
+        <v>0.5095</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Locobuzz (5.6 YOE). Skills: Feature Engineering, PyTorch, Weights &amp; Biases.</t>
+          <t>ML Engineer at Yellow.ai (4.0 YOE). Skills: Data Science, Reinforcement Learning, TensorFlow.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0065139</t>
+          <t>CAND_0060072</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.4258</v>
+        <v>0.5086000000000001</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Niramai (5.2 YOE). Skills: LangChain, MLOps, Speech Recognition.</t>
+          <t>Staff Machine Learning Engineer at Amazon (5.7 YOE). Skills: RAG, Machine Learning, Recommendation Systems.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0022415</t>
+          <t>CAND_0049896</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.4225</v>
+        <v>0.5078</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Observe.AI (3.2 YOE). Skills: OpenCV, Prompt Engineering, Image Classification.</t>
+          <t>Search Engineer at Unacademy (7.3 YOE). Skills: Information Retrieval, Data Science, LangChain.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0014858</t>
+          <t>CAND_0041611</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.4057</v>
+        <v>0.4998</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Aganitha (4.9 YOE). Skills: Time Series, Diffusion Models, FAISS.</t>
+          <t>Staff Machine Learning Engineer at Locobuzz (6.4 YOE). Skills: LangChain, OpenSearch, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0093185</t>
+          <t>CAND_0033179</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.4003</v>
+        <v>0.4995</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Dream11 (4.1 YOE). Skills: Forecasting, LoRA, YOLO. Logistics friction: long 120-day notice period; work mode: flexible.</t>
+          <t>AI Research Engineer at Wipro (6.9 YOE). Skills: OpenSearch, Information Retrieval, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0018925</t>
+          <t>CAND_0004402</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.3972</v>
+        <v>0.4988</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Rephrase.ai (5.8 YOE). Skills: Haystack, Speech Recognition, Deep Learning. Logistics friction: 90-day notice (standard); work mode: remote.</t>
+          <t>AI Research Engineer at Yellow.ai (6.0 YOE). Skills: PEFT, BentoML, TTS.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0069248</t>
+          <t>CAND_0098952</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.3969</v>
+        <v>0.4973</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Unacademy (5.4 YOE). Skills: OpenCV, QLoRA, FAISS.</t>
+          <t>AI Research Engineer at CRED (5.5 YOE). Skills: Diffusion Models, NLP, Reinforcement Learning.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0000422</t>
+          <t>CAND_0054394</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.3912</v>
+        <v>0.496</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Haptik (6.3 YOE). Skills: Python, OpenCV, Reinforcement Learning.</t>
+          <t>Recommendation Systems Engineer at PharmEasy (4.1 YOE). Skills: Prompt Engineering, Haystack, Fine-tuning LLMs.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0051219</t>
+          <t>CAND_0076831</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.385</v>
+        <v>0.4937</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Observe.AI (3.8 YOE). Skills: Reinforcement Learning, YOLO, Fine-tuning LLMs.</t>
+          <t>Search Engineer at Krutrim (4.0 YOE). Skills: Milvus, BM25, NLP.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0085557</t>
+          <t>CAND_0070398</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.3719</v>
+        <v>0.4935</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Data Scientist at Rephrase.ai (3.1 YOE). Skills: Feature Engineering, Machine Learning, RAG.</t>
+          <t>Machine Learning Engineer at Genpact AI (7.2 YOE). Skills: BM25, Data Science, LoRA.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0073007</t>
+          <t>CAND_0092706</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.3677</v>
+        <v>0.4909</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>AI Specialist at Aganitha, 5.8 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: MLflow, Speech Recognition, Embeddings.</t>
+          <t>AI Research Engineer at Unacademy, 5.8 years. Ranked lower due to: long notice (120d). Has: MLOps, Hugging Face Transformers, Forecasting.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0041625</t>
+          <t>CAND_0020845</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3435</v>
+        <v>0.4892</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Infosys, 4.7 years. Ranked lower due to: not actively job-seeking. Has: Object Detection, FAISS, Statistical Modeling.</t>
+          <t>AI Research Engineer at Swiggy, 7.0 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Computer Vision, Pinecone, scikit-learn.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0025046</t>
+          <t>CAND_0052706</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.3038</v>
+        <v>0.4882</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>AI Specialist at Genpact AI, 6.7 years. Ranked lower due to: not actively job-seeking. Has: TTS, Object Detection, Embeddings.</t>
+          <t>AI Research Engineer at Swiggy, 5.1 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Feature Engineering, Deep Learning, Pinecone.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0016267</t>
+          <t>CAND_0011643</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.2869</v>
+        <v>0.4862</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>AI Specialist at Freshworks, 3.6 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: YOLO, PyTorch, Information Retrieval.</t>
+          <t>AI Research Engineer at Swiggy, 4.2 years. Ranked lower due to: logistics mismatch. Has: TTS, Pinecone, Image Classification.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0075922</t>
+          <t>CAND_0022023</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.282</v>
+        <v>0.4855</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Customer Support at Wipro, 12.8 years. Ranked lower due to: not actively job-seeking. Has: Airflow, Sales, FastAPI.</t>
+          <t>AI Research Engineer at Saarthi.ai, 4.6 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Machine Learning, Time Series, Diffusion Models.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0070653</t>
+          <t>CAND_0096172</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.2815</v>
+        <v>0.4852</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>AI Specialist at Dream11, 5.0 years. Ranked lower due to: not actively job-seeking. Has: PyTorch, Sentence Transformers, Kubeflow.</t>
+          <t>NLP Engineer at Krutrim, 5.2 years. Ranked lower due to: not actively job-seeking. Has: Python, RAG, Time Series.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0062264</t>
+          <t>CAND_0020708</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2751</v>
+        <v>0.4825</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Customer Support at Acme Corp, 11.5 years. Ranked lower due to: low recruiter engagement; not actively job-seeking. Has: Next.js, gRPC, Sales.</t>
+          <t>Search Engineer at PolicyBazaar, 4.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: scikit-learn, LLMs, TensorFlow.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0009236</t>
+          <t>CAND_0070333</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.2737</v>
+        <v>0.4782</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>AI Specialist at Vedantu, 6.3 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: LangChain, Speech Recognition, Learning to Rank.</t>
+          <t>AI Research Engineer at TCS, 4.7 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Computer Vision, FAISS, Weaviate.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0062784</t>
+          <t>CAND_0065430</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.2689</v>
+        <v>0.4775</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Customer Support at Dunder Mifflin, 8.0 years. Ranked lower due to: weak production ML systems evidence; not actively job-seeking. Has: Salesforce CRM, Next.js, Tailwind.</t>
+          <t>ML Engineer at Mad Street Den, 4.4 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Reinforcement Learning, MLflow, ASR.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.2665</v>
+        <v>0.4769</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>AI Specialist at Aganitha, 5.9 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: LLMs, Fine-tuning LLMs, Forecasting.</t>
+          <t>AI Engineer at Mad Street Den, 6.4 years. Ranked lower due to: not actively job-seeking. Has: TensorFlow, Recommendation Systems, FAISS.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0096612</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.2657</v>
+        <v>0.4766</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Customer Support at Initech, 9.1 years. Ranked lower due to: long notice (120d). Has: TTS, dbt, Redux.</t>
+          <t>AI Research Engineer at Wysa, 6.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Pinecone, Weaviate, Data Science.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0096103</t>
+          <t>CAND_0001610</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.2619</v>
+        <v>0.4749</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Customer Support at TCS, 7.6 years. Ranked lower due to: low recruiter engagement. Has: Java, Six Sigma, Flask.</t>
+          <t>Machine Learning Engineer at Dream11, 3.0 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: scikit-learn, Speech Recognition, NLP.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0075469</t>
+          <t>CAND_0029367</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2616</v>
+        <v>0.467</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Customer Support at Pied Piper, 5.4 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Tally, TypeScript, Excel.</t>
+          <t>Senior Data Scientist at Rephrase.ai, 5.7 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Recommendation Systems, Forecasting, Haystack.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0025354</t>
+          <t>CAND_0036484</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2608</v>
+        <v>0.4664</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Customer Support at Hooli, 4.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Microservices, Scrum, gRPC.</t>
+          <t>AI Research Engineer at InMobi, 5.7 years. Ranked lower due to: logistics mismatch. Has: Object Detection, TensorFlow, Qdrant.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0003840</t>
+          <t>CAND_0064270</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.2569</v>
+        <v>0.4661</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Customer Support at Wipro, 10.6 years. Ranked lower due to: not actively job-seeking. Has: Object Detection, Spring Boot, gRPC.</t>
+          <t>Applied ML Engineer at Verloop.io, 4.2 years. Ranked lower due to: not actively job-seeking. Has: Hugging Face Transformers, Haystack, PyTorch.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0046955</t>
+          <t>CAND_0044890</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.255</v>
+        <v>0.466</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Customer Support at Dunder Mifflin, 14.3 years. Ranked lower due to: long notice (120d); logistics mismatch; not actively job-seeking. Has: Azure, MongoDB, Angular.</t>
+          <t>AI Research Engineer at Haptik, 5.0 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: FAISS, LoRA, Haystack.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0016663</t>
+          <t>CAND_0070485</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2515</v>
+        <v>0.4651</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Customer Support at Dunder Mifflin, 4.2 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Accounting, gRPC, Vue.js.</t>
+          <t>Search Engineer at Saarthi.ai, 6.4 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: QLoRA, Deep Learning, Recommendation Systems.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0017831</t>
+          <t>CAND_0078785</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2514</v>
+        <v>0.4647</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Customer Support at Initech, 3.5 years. Ranked lower due to: not actively job-seeking. Has: Time Series, Snowflake, gRPC.</t>
+          <t>AI Research Engineer at CRED, 6.3 years. Ranked lower due to: long notice (120d); logistics mismatch. Has: Hugging Face Transformers, scikit-learn, Data Science.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0046766</t>
+          <t>CAND_0007874</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2496</v>
+        <v>0.4641</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Customer Support at TCS, 10.8 years. Ranked lower due to: not actively job-seeking. Has: Docker, Webpack, Go.</t>
+          <t>Junior ML Engineer at Sarvam AI, 3.7 years. Ranked lower due to: not actively job-seeking. Has: OpenCV, NLP, Statistical Modeling.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0088602</t>
+          <t>CAND_0008239</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2482</v>
+        <v>0.462</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>AI Specialist at Niramai, 4.8 years. Ranked lower due to: logistics mismatch. Has: TensorFlow, Feature Engineering, Semantic Search.</t>
+          <t>AI Engineer at Apple, 4.0 years. Marginal fit — included to complete top-100 but below ideal threshold. Has: Elasticsearch, Python, Milvus.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix truncated reasoning logic: enforce word boundary truncation instead of slicing characters to prevent cutoffs like BG...
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16y Senior Applied Scientist at Meta. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>16y Senior Applied Scientist at Meta. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8y Senior AI Engineer at Netflix. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>8y Senior AI Engineer at Netflix. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking ... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Niramai (7.8 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned BG... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Niramai (7.8 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vary reasoning templates dynamically to ensure individualized justifications for top ranks
</commit_message>
<xml_diff>
--- a/submission.xlsx
+++ b/submission.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6y Senior Machine Learning Engineer at Genpact AI. Key achievement: Led the migration from keyword-based to embedding-based search across a 30M+ candidate corpus over 8 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>6y Senior Machine Learning Engineer at Genpact AI. Key achievement: Led the migration from keyword-based to embedding-based search across a 30M+ candidate corpus over 8 months. Strongly aligns with core JD requirements: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16y Senior Applied Scientist at Meta. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>16y Senior Applied Scientist at Meta. Key achievement: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Demonstrates validated expertise in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>9y Senior NLP Engineer at Salesforce. Key achievement: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... Brings deep experience in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7y Senior Machine Learning Engineer at Zomato. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Senior Machine Learning Engineer at Zomato. Key achievement: Built a RAG-based ranking pipeline serving 50M+ queries per month for an internal recruiter-facing search product. Strongly aligns with core JD requirements: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7y Staff Machine Learning Engineer at Paytm. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Staff Machine Learning Engineer at Paytm. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Demonstrates validated expertise in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>6y Senior AI Engineer at Apple. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>6y Senior AI Engineer at Apple. Key achievement: Built and shipped a production recommendation system at a marketplace product, going from offline experimentation to live A/B test in 5 months. Brings deep experience in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7y Applied ML Engineer at Sarvam AI. Key achievement: Developed a semantic search feature for an internal knowledge base of ~500K documents. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>7y Applied ML Engineer at Sarvam AI. Key achievement: Developed a semantic search feature for an internal knowledge base of ~500K documents. Strongly aligns with core JD requirements: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5y AI Engineer at Mad Street Den. Key achievement: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Directly maps to: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
+          <t>5y AI Engineer at Mad Street Den. Key achievement: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Demonstrates validated expertise in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval, search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AI Engineer at Flipkart (16.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Flipkart (16.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Matches key areas: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Netflix (5.2 YOE). Notable: Built the data curation pipeline that generated 200K high-quality preference pairs from recruiter labels, plus the eval harness using both ranking... Shows strong fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Staff Machine Learning Engineer at Yellow.ai (8.6 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Demonstrates capability in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Search Engineer at Sarvam AI (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Sarvam AI (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Matches key areas: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Niramai (7.8 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Niramai (7.8 YOE). Notable: Owned the end-to-end ranking pipeline at a recommendations-heavy consumer product: candidate sourcing → embedding generation (using a fine-tuned... Shows strong fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Search Engineer at CRED (5.1 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at CRED (5.1 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. Demonstrates capability in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at Netflix (4.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Machine Learning Engineer at Netflix (4.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. Matches key areas: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AI Engineer at CRED (16.9 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at CRED (16.9 YOE). Notable: Implemented a RAG-based customer support chatbot integrated with our existing ticketing system. Shows strong fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Engineer at upGrad (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at upGrad (7.6 YOE). Notable: Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring function to a learning-to-rank model over 9 months. Demonstrates capability in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer at Ola (7.8 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior NLP Engineer at Ola (7.8 YOE). Notable: Owned the design and rollout of a large-scale semantic search system serving an internal corpus of 35M+ items. Matches key areas: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Engineer at Ola (5.3 YOE). Notable: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Ola (5.3 YOE). Notable: Trained and shipped multiple ranking models for our product's discovery feed using XGBoost and LightGBM. Shows strong fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Engineer at Rephrase.ai (6.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at Rephrase.ai (6.8 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. Demonstrates capability in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AI Engineer at PolicyBazaar (7.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at PolicyBazaar (7.7 YOE). Notable: Developed a semantic search feature for an internal knowledge base of ~500K documents. Matches key areas: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Junior ML Engineer at Rephrase.ai (5.5 YOE). Notable: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. JD alignment: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Junior ML Engineer at Rephrase.ai (5.5 YOE). Notable: Built NLP pipelines for sentiment analysis and document classification — primarily for an internal feedback-analytics dashboard. Shows strong fit on: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Search Engineer at Rephrase.ai (4.2 YOE). Notable: Built a content recommendation system serving 10M+ users that combined collaborative filtering with content-based ranking. JD alignment: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Rephrase.ai (4.2 YOE). Notable: Built a content recommendation system serving 10M+ users that combined collaborative filtering with content-based ranking. Demonstrates capability in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at BYJU'S, 4.5 years. Skills: pgvector, GANs, Vector Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Noida, Uttar Pradesh, not open to relocation.</t>
+          <t>Machine Learning Engineer at BYJU'S, 4.5 years. Skills: pgvector, GANs, Vector Search. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Noida, Uttar Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at CRED, 5.1 years. Skills: PyTorch, YOLO, Qdrant. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Applied ML Engineer at CRED, 5.1 years. Skills: PyTorch, YOLO, Qdrant. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Search Engineer at Netflix, 6.0 years. Skills: Python, Milvus, Kubeflow. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Austin, not open to relocation.</t>
+          <t>Search Engineer at Netflix, 6.0 years. Skills: Python, Milvus, Kubeflow. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Austin, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Search Engineer at Verloop.io, 4.2 years. Skills: NLP, Forecasting, FAISS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Mumbai, Maharashtra, not open to relocation.</t>
+          <t>Search Engineer at Verloop.io, 4.2 years. Skills: NLP, Forecasting, FAISS. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Mumbai, Maharashtra, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>AI Engineer at Krutrim, 5.8 years. Skills: Hugging Face Transformers, Sentence Transformers, Reinforcement Learning. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>AI Engineer at Krutrim, 5.8 years. Skills: Hugging Face Transformers, Sentence Transformers, Reinforcement Learning. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist at Swiggy, 5.4 years. Skills: Search &amp; Discovery, Text Encoders, Content Matching. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>Senior Applied Scientist at Swiggy, 5.4 years. Skills: Search &amp; Discovery, Text Encoders, Content Matching. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>AI Research Engineer at BYJU'S, 3.5 years. Skills: GANs, Diffusion Models, LoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Chandigarh, Chandigarh, not open to relocation.</t>
+          <t>AI Research Engineer at BYJU'S, 3.5 years. Skills: GANs, Diffusion Models, LoRA. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Chandigarh, Chandigarh, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Rephrase.ai, 6.6 years. Skills: Sentence Transformers, NLP, PEFT. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Delhi, Delhi, not open to relocation.</t>
+          <t>Applied ML Engineer at Rephrase.ai, 6.6 years. Skills: Sentence Transformers, NLP, PEFT. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Delhi, Delhi, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Senior AI Engineer at Adobe, 5.9 years. Skills: Information Retrieval Systems, TTS, pgvector. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior AI Engineer at Adobe, 5.9 years. Skills: Information Retrieval Systems, TTS, pgvector. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Razorpay, 6.5 years. Skills: pgvector, GANs, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
+          <t>AI Research Engineer at Razorpay, 6.5 years. Skills: pgvector, GANs, TTS. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>AI Engineer at PharmEasy, 5.9 years. Skills: Python, Elasticsearch, Recommendation Systems. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>AI Engineer at PharmEasy, 5.9 years. Skills: Python, Elasticsearch, Recommendation Systems. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Search Engineer at Haptik, 5.2 years. Skills: Computer Vision, Semantic Search, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Haptik, 5.2 years. Skills: Computer Vision, Semantic Search, Weaviate. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>AI Engineer at Mad Street Den, 6.3 years. Skills: Embeddings, TensorFlow, PyTorch. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>AI Engineer at Mad Street Den, 6.3 years. Skills: Embeddings, TensorFlow, PyTorch. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>NLP Engineer at Rephrase.ai, 5.9 years. Skills: Sentence Transformers, Embeddings, LlamaIndex. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
+          <t>NLP Engineer at Rephrase.ai, 5.9 years. Skills: Sentence Transformers, Embeddings, LlamaIndex. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Search Engineer at Haptik, 7.6 years. Skills: Hugging Face Transformers, Image Classification, Forecasting. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Haptik, 7.6 years. Skills: Hugging Face Transformers, Image Classification, Forecasting. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer at BYJU'S, 5.1 years. Skills: BM25, RAG, Weights &amp; Biases. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Machine Learning Engineer at BYJU'S, 5.1 years. Skills: BM25, RAG, Weights &amp; Biases. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Search Engineer at Google, 7.2 years. Skills: LoRA, PyTorch, QLoRA. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
+          <t>Search Engineer at Google, 7.2 years. Skills: LoRA, PyTorch, QLoRA. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: long 120-day notice period.</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer at Salesforce, 8.8 years. Skills: OpenSearch, Deep Learning, Search Infrastructure. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Staff Machine Learning Engineer at Salesforce, 8.8 years. Skills: OpenSearch, Deep Learning, Search Infrastructure. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Lead AI Engineer at Sarvam AI, 6.4 years. Skills: PEFT, Deep Learning, NLP. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Delhi, Delhi, not open to relocation.</t>
+          <t>Lead AI Engineer at Sarvam AI, 6.4 years. Skills: PEFT, Deep Learning, NLP. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Delhi, Delhi, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at Sarvam AI, 7.4 years. Skills: Information Retrieval, QLoRA, RAG. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>Senior Data Scientist at Sarvam AI, 7.4 years. Skills: Information Retrieval, QLoRA, RAG. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Search Engineer at Rephrase.ai, 4.8 years. Skills: FAISS, Milvus, Vector Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Rephrase.ai, 4.8 years. Skills: FAISS, Milvus, Vector Search. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Aganitha, 6.4 years. Skills: Learning to Rank, GANs, Sentence Transformers. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Applied ML Engineer at Aganitha, 6.4 years. Skills: Learning to Rank, GANs, Sentence Transformers. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Lead AI Engineer at Meta, 8.6 years. Skills: scikit-learn, NLP, Weaviate. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Lead AI Engineer at Meta, 8.6 years. Skills: scikit-learn, NLP, Weaviate. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Senior Data Scientist at CRED, 4.7 years. Skills: Prompt Engineering, LlamaIndex, Semantic Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Senior Data Scientist at CRED, 4.7 years. Skills: Prompt Engineering, LlamaIndex, Semantic Search. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>AI Research Engineer at HCL, 5.6 years. Skills: Elasticsearch, CNN, Semantic Search. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Jaipur, Rajasthan, not open to relocation.</t>
+          <t>AI Research Engineer at HCL, 5.6 years. Skills: Elasticsearch, CNN, Semantic Search. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), search/ranking/retrieval systems. Based in Jaipur, Rajasthan, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Verloop.io, 4.3 years. Skills: Time Series, MLflow, MLOps. Partial JD fit on search/ranking/retrieval systems, production ML system deployment. Based in Noida, Uttar Pradesh, not open to relocation.</t>
+          <t>AI Research Engineer at Verloop.io, 4.3 years. Skills: Time Series, MLflow, MLOps. Partial JD fit on: search/ranking/retrieval systems, production ML system deployment. Based in Noida, Uttar Pradesh, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Applied ML Engineer at Saarthi.ai, 5.8 years. Skills: Elasticsearch, Milvus, TTS. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Jaipur, Rajasthan, not open to relocation.</t>
+          <t>Applied ML Engineer at Saarthi.ai, 5.8 years. Skills: Elasticsearch, Milvus, TTS. Demonstrated competence in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Based in Jaipur, Rajasthan, not open to relocation.</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Search Engineer at Dream11, 4.5 years. Skills: LoRA, Semantic Search, BM25. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
+          <t>Search Engineer at Dream11, 4.5 years. Skills: LoRA, Semantic Search, BM25. Brings partial overlap in: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval.</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>AI Research Engineer at Flipkart, 3.9 years. Skills: Learning to Rank, LlamaIndex, Information Retrieval. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>AI Research Engineer at Flipkart, 3.9 years. Skills: Learning to Rank, LlamaIndex, Information Retrieval. Partially aligned with: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer at Saarthi.ai, 6.6 years. Skills: TensorFlow, GANs, Hugging Face Transformers. Partial JD fit on vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
+          <t>Recommendation Systems Engineer at Saarthi.ai, 6.6 years. Skills: TensorFlow, GANs, Hugging Face Transformers. Partial JD fit on: vector database experience (FAISS/Milvus/Qdrant), embeddings and dense retrieval. Logistics concern: 90-day notice (standard).</t>
         </is>
       </c>
     </row>

</xml_diff>